<commit_message>
Complete Task 4 forecasting analysis
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_unified_data_enriched.xlsx
+++ b/data/processed/ethiopia_fi_unified_data_enriched.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI64"/>
+  <dimension ref="A1:AI67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7438,6 +7438,315 @@
       </c>
       <c r="AI64" t="inlineStr"/>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>REC_0062</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>USAGE</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Made or Received Digital Payment</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>USG_DIGITAL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="n">
+        <v>12</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2017-12-31</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>World Bank Blog (Findex 2017 Ethiopia takeaways)</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>survey</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>https://blogs.worldbank.org/en/africacan/financial-inclusion-in-ethiopia-10-takeaways-from-findex-2017</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr"/>
+      <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr"/>
+      <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>Made or received digital payments in the past year (%) ... 12</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>Fills Usage target series gap for Task 4 forecasting; Ethiopia-specific Findex 2017 figure</t>
+        </is>
+      </c>
+      <c r="AI65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>REC_0063</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>USAGE</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Made or Received Digital Payment</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>USG_DIGITAL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>20</v>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2021-12-31</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>World Bank Blog (Ethiopia mobile/account usage)</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>survey</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>https://blogs.worldbank.org/en/africacan/mobile-phone-technology-could-expand-equitable-access-financial-services-ethiopia</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
+      <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr"/>
+      <c r="AB66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr"/>
+      <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>20% of adults—used their accounts for digital payments</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
+          <t>Fills Usage target series gap for Task 4 forecasting; Ethiopia-specific Findex 2021 figure</t>
+        </is>
+      </c>
+      <c r="AI66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>REC_0064</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>USAGE</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Made or Received Digital Payment</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>USG_DIGITAL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="n">
+        <v>35</v>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>10Academy Week 11 Challenge Document</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>survey</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>internal_challenge_doc</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr"/>
+      <c r="X67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr"/>
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr"/>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr"/>
+      <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t>Made or received digital payment: ~35%</t>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
+          <t>Approximate figure as stated in challenge doc overview; not independently re-verified against primary Findex 2024 source</t>
+        </is>
+      </c>
+      <c r="AI67" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>